<commit_message>
chore: update browser cache, sessions, and indexedDB data for scraper
</commit_message>
<xml_diff>
--- a/Colombia/Resultados electorales.xlsx
+++ b/Colombia/Resultados electorales.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\juansoag\Downloads\Github\Avances_tesis\Colombia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{660A83B6-8F22-4201-B938-9D9F000E5E5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23D2A309-E7AD-4261-9EBE-2ECBE856141A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20370" yWindow="1245" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Candidatos E-26 ALC" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5011" uniqueCount="1431">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5003" uniqueCount="1423">
   <si>
     <t>ID Candidato</t>
   </si>
@@ -3768,18 +3768,6 @@
     <t>https://www.facebook.com/Robertojimenezdosquebradas</t>
   </si>
   <si>
-    <t>https://www.facebook.com/jorgenavasgranados/?locale=es_LA</t>
-  </si>
-  <si>
-    <t>https://www.tiktok.com/@jorge_navas</t>
-  </si>
-  <si>
-    <t>https://x.com/JorgeANavasG</t>
-  </si>
-  <si>
-    <t>https://www.instagram.com/jorgenavasgranados/</t>
-  </si>
-  <si>
     <t>https://www.facebook.com/joseluisosoriogalviis/mentions/</t>
   </si>
   <si>
@@ -4243,18 +4231,6 @@
   </si>
   <si>
     <t>https://www.facebook.com/linamardearmas/?locale=es_LA</t>
-  </si>
-  <si>
-    <t>https://www.facebook.com/wilsongonzalezpiedecuesta/</t>
-  </si>
-  <si>
-    <t>https://www.instagram.com/wilsongonzalezv_/</t>
-  </si>
-  <si>
-    <t>https://www.tiktok.com/@wilsongonzalezv_</t>
-  </si>
-  <si>
-    <t>https://x.com/wilsongonzale_</t>
   </si>
   <si>
     <t>https://www.instagram.com/rodolfo.correav/</t>
@@ -4342,7 +4318,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4404,6 +4380,13 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="7">
@@ -4478,7 +4461,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -4568,12 +4551,17 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -12604,7 +12592,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="267" spans="1:9" s="36" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A267" s="2" t="s">
         <v>736</v>
       </c>
@@ -15117,10 +15105,10 @@
         <v>1213</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>1414</v>
+        <v>1406</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>1416</v>
+        <v>1408</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>934</v>
@@ -15199,14 +15187,14 @@
       <c r="H3" s="2"/>
       <c r="I3" s="2"/>
       <c r="J3" s="21" t="s">
-        <v>1266</v>
+        <v>1262</v>
       </c>
       <c r="K3" s="21" t="s">
-        <v>1267</v>
+        <v>1263</v>
       </c>
       <c r="L3" s="16"/>
       <c r="M3" s="21" t="s">
-        <v>1268</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -15579,16 +15567,16 @@
       <c r="H15" s="5"/>
       <c r="I15" s="5"/>
       <c r="J15" s="22" t="s">
-        <v>1380</v>
+        <v>1376</v>
       </c>
       <c r="K15" s="22" t="s">
-        <v>1381</v>
+        <v>1377</v>
       </c>
       <c r="L15" s="22" t="s">
-        <v>1382</v>
+        <v>1378</v>
       </c>
       <c r="M15" s="22" t="s">
-        <v>1379</v>
+        <v>1375</v>
       </c>
     </row>
     <row r="16" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -16023,16 +16011,16 @@
       <c r="H29" s="5"/>
       <c r="I29" s="5"/>
       <c r="J29" s="22" t="s">
-        <v>1315</v>
+        <v>1311</v>
       </c>
       <c r="K29" s="22" t="s">
-        <v>1316</v>
+        <v>1312</v>
       </c>
       <c r="L29" s="22" t="s">
-        <v>1317</v>
+        <v>1313</v>
       </c>
       <c r="M29" s="22" t="s">
-        <v>1318</v>
+        <v>1314</v>
       </c>
     </row>
     <row r="30" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -16407,12 +16395,12 @@
       <c r="H41" s="2"/>
       <c r="I41" s="2"/>
       <c r="J41" s="21" t="s">
-        <v>1297</v>
+        <v>1293</v>
       </c>
       <c r="K41" s="16"/>
       <c r="L41" s="16"/>
       <c r="M41" s="21" t="s">
-        <v>1425</v>
+        <v>1417</v>
       </c>
     </row>
     <row r="42" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -16610,7 +16598,7 @@
       <c r="K47" s="17"/>
       <c r="L47" s="17"/>
       <c r="M47" s="22" t="s">
-        <v>1387</v>
+        <v>1383</v>
       </c>
     </row>
     <row r="48" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -17085,13 +17073,13 @@
       <c r="H61" s="5"/>
       <c r="I61" s="5"/>
       <c r="J61" s="22" t="s">
-        <v>1340</v>
+        <v>1336</v>
       </c>
       <c r="K61" s="22" t="s">
-        <v>1339</v>
+        <v>1335</v>
       </c>
       <c r="L61" s="22" t="s">
-        <v>1341</v>
+        <v>1337</v>
       </c>
       <c r="M61" s="17"/>
     </row>
@@ -17121,16 +17109,16 @@
       <c r="H62" s="2"/>
       <c r="I62" s="2"/>
       <c r="J62" s="21" t="s">
-        <v>1418</v>
+        <v>1410</v>
       </c>
       <c r="K62" s="21" t="s">
-        <v>1420</v>
+        <v>1412</v>
       </c>
       <c r="L62" s="21" t="s">
-        <v>1421</v>
+        <v>1413</v>
       </c>
       <c r="M62" s="21" t="s">
-        <v>1419</v>
+        <v>1411</v>
       </c>
     </row>
     <row r="63" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -17273,16 +17261,16 @@
       <c r="H66" s="5"/>
       <c r="I66" s="5"/>
       <c r="J66" s="22" t="s">
-        <v>1249</v>
+        <v>1245</v>
       </c>
       <c r="K66" s="22" t="s">
-        <v>1251</v>
+        <v>1247</v>
       </c>
       <c r="L66" s="22" t="s">
-        <v>1250</v>
+        <v>1246</v>
       </c>
       <c r="M66" s="22" t="s">
-        <v>1252</v>
+        <v>1248</v>
       </c>
     </row>
     <row r="67" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -17311,16 +17299,16 @@
       <c r="H67" s="5"/>
       <c r="I67" s="5"/>
       <c r="J67" s="22" t="s">
-        <v>1258</v>
+        <v>1254</v>
       </c>
       <c r="K67" s="22" t="s">
-        <v>1260</v>
+        <v>1256</v>
       </c>
       <c r="L67" s="22" t="s">
-        <v>1259</v>
+        <v>1255</v>
       </c>
       <c r="M67" s="22" t="s">
-        <v>1261</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="68" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -17349,16 +17337,16 @@
       <c r="H68" s="5"/>
       <c r="I68" s="5"/>
       <c r="J68" s="22" t="s">
-        <v>1408</v>
+        <v>1400</v>
       </c>
       <c r="K68" s="22" t="s">
-        <v>1410</v>
+        <v>1402</v>
       </c>
       <c r="L68" s="22" t="s">
-        <v>1411</v>
+        <v>1403</v>
       </c>
       <c r="M68" s="22" t="s">
-        <v>1409</v>
+        <v>1401</v>
       </c>
     </row>
     <row r="69" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -17387,12 +17375,12 @@
       <c r="H69" s="2"/>
       <c r="I69" s="2"/>
       <c r="J69" s="21" t="s">
-        <v>1412</v>
+        <v>1404</v>
       </c>
       <c r="K69" s="16"/>
       <c r="L69" s="16"/>
       <c r="M69" s="21" t="s">
-        <v>1413</v>
+        <v>1405</v>
       </c>
     </row>
     <row r="70" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -17699,16 +17687,16 @@
       <c r="H79" s="5"/>
       <c r="I79" s="5"/>
       <c r="J79" s="22" t="s">
-        <v>1254</v>
+        <v>1250</v>
       </c>
       <c r="K79" s="22" t="s">
-        <v>1286</v>
+        <v>1282</v>
       </c>
       <c r="L79" s="22" t="s">
-        <v>1287</v>
+        <v>1283</v>
       </c>
       <c r="M79" s="22" t="s">
-        <v>1285</v>
+        <v>1281</v>
       </c>
     </row>
     <row r="80" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -17977,7 +17965,7 @@
       <c r="H88" s="5"/>
       <c r="I88" s="5"/>
       <c r="J88" s="17"/>
-      <c r="K88" s="35"/>
+      <c r="K88" s="33"/>
       <c r="L88" s="17"/>
       <c r="M88" s="17"/>
     </row>
@@ -18309,16 +18297,16 @@
       <c r="H98" s="5"/>
       <c r="I98" s="5"/>
       <c r="J98" s="22" t="s">
-        <v>1422</v>
+        <v>1414</v>
       </c>
       <c r="K98" s="22" t="s">
-        <v>1424</v>
+        <v>1416</v>
       </c>
       <c r="L98" s="22" t="s">
-        <v>1423</v>
+        <v>1415</v>
       </c>
       <c r="M98" s="22" t="s">
-        <v>1296</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="99" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -18347,16 +18335,16 @@
       <c r="H99" s="5"/>
       <c r="I99" s="5"/>
       <c r="J99" s="22" t="s">
-        <v>1388</v>
+        <v>1384</v>
       </c>
       <c r="K99" s="22" t="s">
-        <v>1389</v>
+        <v>1385</v>
       </c>
       <c r="L99" s="22" t="s">
-        <v>1391</v>
+        <v>1387</v>
       </c>
       <c r="M99" s="22" t="s">
-        <v>1390</v>
+        <v>1386</v>
       </c>
     </row>
     <row r="100" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -18657,16 +18645,16 @@
       <c r="H108" s="2"/>
       <c r="I108" s="2"/>
       <c r="J108" s="21" t="s">
-        <v>1247</v>
+        <v>1243</v>
       </c>
       <c r="K108" s="21" t="s">
-        <v>1246</v>
+        <v>1242</v>
       </c>
       <c r="L108" s="21" t="s">
-        <v>1248</v>
+        <v>1244</v>
       </c>
       <c r="M108" s="21" t="s">
-        <v>1245</v>
+        <v>1241</v>
       </c>
     </row>
     <row r="109" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -19019,16 +19007,16 @@
       <c r="H119" s="2"/>
       <c r="I119" s="2"/>
       <c r="J119" s="21" t="s">
-        <v>1311</v>
+        <v>1307</v>
       </c>
       <c r="K119" s="21" t="s">
-        <v>1312</v>
+        <v>1308</v>
       </c>
       <c r="L119" s="21" t="s">
-        <v>1313</v>
+        <v>1309</v>
       </c>
       <c r="M119" s="21" t="s">
-        <v>1314</v>
+        <v>1310</v>
       </c>
     </row>
     <row r="120" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -19057,16 +19045,16 @@
       <c r="H120" s="5"/>
       <c r="I120" s="5"/>
       <c r="J120" s="22" t="s">
-        <v>1360</v>
+        <v>1356</v>
       </c>
       <c r="K120" s="22" t="s">
-        <v>1361</v>
+        <v>1357</v>
       </c>
       <c r="L120" s="22" t="s">
-        <v>1362</v>
+        <v>1358</v>
       </c>
       <c r="M120" s="22" t="s">
-        <v>1363</v>
+        <v>1359</v>
       </c>
     </row>
     <row r="121" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -19095,16 +19083,16 @@
       <c r="H121" s="5"/>
       <c r="I121" s="5"/>
       <c r="J121" s="22" t="s">
-        <v>1371</v>
+        <v>1367</v>
       </c>
       <c r="K121" s="22" t="s">
-        <v>1372</v>
+        <v>1368</v>
       </c>
       <c r="L121" s="22" t="s">
-        <v>1373</v>
+        <v>1369</v>
       </c>
       <c r="M121" s="22" t="s">
-        <v>1374</v>
+        <v>1370</v>
       </c>
     </row>
     <row r="122" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -19412,16 +19400,16 @@
       <c r="H131" s="2"/>
       <c r="I131" s="2"/>
       <c r="J131" s="21" t="s">
+        <v>1249</v>
+      </c>
+      <c r="K131" s="21" t="s">
+        <v>1252</v>
+      </c>
+      <c r="L131" s="21" t="s">
+        <v>1251</v>
+      </c>
+      <c r="M131" s="21" t="s">
         <v>1253</v>
-      </c>
-      <c r="K131" s="21" t="s">
-        <v>1256</v>
-      </c>
-      <c r="L131" s="21" t="s">
-        <v>1255</v>
-      </c>
-      <c r="M131" s="21" t="s">
-        <v>1257</v>
       </c>
     </row>
     <row r="132" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -19450,16 +19438,16 @@
       <c r="H132" s="5"/>
       <c r="I132" s="5"/>
       <c r="J132" s="22" t="s">
-        <v>1277</v>
+        <v>1273</v>
       </c>
       <c r="K132" s="22" t="s">
-        <v>1278</v>
+        <v>1274</v>
       </c>
       <c r="L132" s="22" t="s">
-        <v>1279</v>
+        <v>1275</v>
       </c>
       <c r="M132" s="22" t="s">
-        <v>1280</v>
+        <v>1276</v>
       </c>
     </row>
     <row r="133" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -19620,12 +19608,12 @@
       <c r="H137" s="5"/>
       <c r="I137" s="5"/>
       <c r="J137" s="22" t="s">
-        <v>1324</v>
+        <v>1320</v>
       </c>
       <c r="K137" s="17"/>
       <c r="L137" s="17"/>
       <c r="M137" s="22" t="s">
-        <v>1325</v>
+        <v>1321</v>
       </c>
     </row>
     <row r="138" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -19760,16 +19748,16 @@
       <c r="H141" s="5"/>
       <c r="I141" s="5"/>
       <c r="J141" s="22" t="s">
+        <v>1348</v>
+      </c>
+      <c r="K141" s="22" t="s">
+        <v>1350</v>
+      </c>
+      <c r="L141" s="22" t="s">
+        <v>1351</v>
+      </c>
+      <c r="M141" s="22" t="s">
         <v>1352</v>
-      </c>
-      <c r="K141" s="22" t="s">
-        <v>1354</v>
-      </c>
-      <c r="L141" s="22" t="s">
-        <v>1355</v>
-      </c>
-      <c r="M141" s="22" t="s">
-        <v>1356</v>
       </c>
     </row>
     <row r="142" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -20084,16 +20072,16 @@
       <c r="H151" s="2"/>
       <c r="I151" s="2"/>
       <c r="J151" s="21" t="s">
-        <v>1281</v>
+        <v>1277</v>
       </c>
       <c r="K151" s="21" t="s">
-        <v>1282</v>
+        <v>1278</v>
       </c>
       <c r="L151" s="21" t="s">
-        <v>1283</v>
+        <v>1279</v>
       </c>
       <c r="M151" s="21" t="s">
-        <v>1284</v>
+        <v>1280</v>
       </c>
     </row>
     <row r="152" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -20122,16 +20110,16 @@
       <c r="H152" s="5"/>
       <c r="I152" s="5"/>
       <c r="J152" s="22" t="s">
-        <v>1300</v>
+        <v>1296</v>
       </c>
       <c r="K152" s="22" t="s">
-        <v>1299</v>
+        <v>1295</v>
       </c>
       <c r="L152" s="22" t="s">
-        <v>1301</v>
+        <v>1297</v>
       </c>
       <c r="M152" s="22" t="s">
-        <v>1298</v>
+        <v>1294</v>
       </c>
     </row>
     <row r="153" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -20160,16 +20148,16 @@
       <c r="H153" s="5"/>
       <c r="I153" s="5"/>
       <c r="J153" s="22" t="s">
+        <v>1315</v>
+      </c>
+      <c r="K153" s="22" t="s">
+        <v>1317</v>
+      </c>
+      <c r="L153" s="22" t="s">
+        <v>1318</v>
+      </c>
+      <c r="M153" s="22" t="s">
         <v>1319</v>
-      </c>
-      <c r="K153" s="22" t="s">
-        <v>1321</v>
-      </c>
-      <c r="L153" s="22" t="s">
-        <v>1322</v>
-      </c>
-      <c r="M153" s="22" t="s">
-        <v>1323</v>
       </c>
     </row>
     <row r="154" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -20198,16 +20186,16 @@
       <c r="H154" s="5"/>
       <c r="I154" s="5"/>
       <c r="J154" s="22" t="s">
-        <v>1392</v>
+        <v>1388</v>
       </c>
       <c r="K154" s="22" t="s">
-        <v>1393</v>
+        <v>1389</v>
       </c>
       <c r="L154" s="22" t="s">
-        <v>1394</v>
+        <v>1390</v>
       </c>
       <c r="M154" s="22" t="s">
-        <v>1395</v>
+        <v>1391</v>
       </c>
     </row>
     <row r="155" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -20628,16 +20616,16 @@
       <c r="H167" s="5"/>
       <c r="I167" s="5"/>
       <c r="J167" s="22" t="s">
-        <v>1262</v>
+        <v>1258</v>
       </c>
       <c r="K167" s="22" t="s">
-        <v>1263</v>
+        <v>1259</v>
       </c>
       <c r="L167" s="22" t="s">
-        <v>1264</v>
+        <v>1260</v>
       </c>
       <c r="M167" s="22" t="s">
-        <v>1265</v>
+        <v>1261</v>
       </c>
     </row>
     <row r="168" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -21020,16 +21008,16 @@
       <c r="H179" s="2"/>
       <c r="I179" s="2"/>
       <c r="J179" s="21" t="s">
-        <v>1335</v>
+        <v>1331</v>
       </c>
       <c r="K179" s="21" t="s">
-        <v>1357</v>
+        <v>1353</v>
       </c>
       <c r="L179" s="21" t="s">
-        <v>1358</v>
+        <v>1354</v>
       </c>
       <c r="M179" s="21" t="s">
-        <v>1359</v>
+        <v>1355</v>
       </c>
     </row>
     <row r="180" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -21058,16 +21046,16 @@
       <c r="H180" s="5"/>
       <c r="I180" s="5"/>
       <c r="J180" s="22" t="s">
-        <v>1375</v>
+        <v>1371</v>
       </c>
       <c r="K180" s="22" t="s">
-        <v>1376</v>
+        <v>1372</v>
       </c>
       <c r="L180" s="22" t="s">
-        <v>1377</v>
+        <v>1373</v>
       </c>
       <c r="M180" s="22" t="s">
-        <v>1378</v>
+        <v>1374</v>
       </c>
     </row>
     <row r="181" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -21096,16 +21084,16 @@
       <c r="H181" s="5"/>
       <c r="I181" s="5"/>
       <c r="J181" s="22" t="s">
-        <v>1404</v>
+        <v>1396</v>
       </c>
       <c r="K181" s="22" t="s">
-        <v>1405</v>
+        <v>1397</v>
       </c>
       <c r="L181" s="22" t="s">
-        <v>1406</v>
+        <v>1398</v>
       </c>
       <c r="M181" s="22" t="s">
-        <v>1407</v>
+        <v>1399</v>
       </c>
     </row>
     <row r="182" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -21668,12 +21656,12 @@
       <c r="H199" s="2"/>
       <c r="I199" s="2"/>
       <c r="J199" s="21" t="s">
-        <v>1306</v>
+        <v>1302</v>
       </c>
       <c r="K199" s="16"/>
       <c r="L199" s="16"/>
       <c r="M199" s="21" t="s">
-        <v>1307</v>
+        <v>1303</v>
       </c>
     </row>
     <row r="200" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -21702,12 +21690,12 @@
       <c r="H200" s="5"/>
       <c r="I200" s="5"/>
       <c r="J200" s="22" t="s">
-        <v>1342</v>
+        <v>1338</v>
       </c>
       <c r="K200" s="17"/>
       <c r="L200" s="17"/>
       <c r="M200" s="22" t="s">
-        <v>1343</v>
+        <v>1339</v>
       </c>
     </row>
     <row r="201" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -21736,16 +21724,16 @@
       <c r="H201" s="5"/>
       <c r="I201" s="5"/>
       <c r="J201" s="22" t="s">
-        <v>1351</v>
+        <v>1347</v>
       </c>
       <c r="K201" s="22" t="s">
-        <v>1349</v>
+        <v>1345</v>
       </c>
       <c r="L201" s="22" t="s">
-        <v>1350</v>
+        <v>1346</v>
       </c>
       <c r="M201" s="22" t="s">
-        <v>1348</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="202" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -21774,14 +21762,14 @@
       <c r="H202" s="5"/>
       <c r="I202" s="5"/>
       <c r="J202" s="22" t="s">
-        <v>1320</v>
+        <v>1316</v>
       </c>
       <c r="K202" s="17"/>
       <c r="L202" s="22" t="s">
-        <v>1364</v>
+        <v>1360</v>
       </c>
       <c r="M202" s="22" t="s">
-        <v>1365</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="203" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -21810,16 +21798,16 @@
       <c r="H203" s="5"/>
       <c r="I203" s="5"/>
       <c r="J203" s="22" t="s">
-        <v>1367</v>
+        <v>1363</v>
       </c>
       <c r="K203" s="22" t="s">
-        <v>1368</v>
+        <v>1364</v>
       </c>
       <c r="L203" s="22" t="s">
-        <v>1369</v>
+        <v>1365</v>
       </c>
       <c r="M203" s="22" t="s">
-        <v>1370</v>
+        <v>1366</v>
       </c>
     </row>
     <row r="204" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -22014,16 +22002,16 @@
       <c r="H209" s="5"/>
       <c r="I209" s="5"/>
       <c r="J209" s="22" t="s">
-        <v>1302</v>
+        <v>1298</v>
       </c>
       <c r="K209" s="22" t="s">
-        <v>1303</v>
+        <v>1299</v>
       </c>
       <c r="L209" s="22" t="s">
-        <v>1304</v>
+        <v>1300</v>
       </c>
       <c r="M209" s="22" t="s">
-        <v>1305</v>
+        <v>1301</v>
       </c>
     </row>
     <row r="210" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -22338,16 +22326,16 @@
       <c r="H219" s="5"/>
       <c r="I219" s="5"/>
       <c r="J219" s="22" t="s">
-        <v>1330</v>
+        <v>1326</v>
       </c>
       <c r="K219" s="22" t="s">
-        <v>1331</v>
+        <v>1327</v>
       </c>
       <c r="L219" s="22" t="s">
-        <v>1332</v>
+        <v>1328</v>
       </c>
       <c r="M219" s="22" t="s">
-        <v>1333</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="220" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -22670,16 +22658,16 @@
       <c r="H229" s="2"/>
       <c r="I229" s="2"/>
       <c r="J229" s="21" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="K229" s="21" t="s">
-        <v>1346</v>
+        <v>1342</v>
       </c>
       <c r="L229" s="21" t="s">
-        <v>1345</v>
+        <v>1341</v>
       </c>
       <c r="M229" s="21" t="s">
-        <v>1347</v>
+        <v>1343</v>
       </c>
     </row>
     <row r="230" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -22796,10 +22784,10 @@
         <v>1</v>
       </c>
       <c r="H233" s="8" t="s">
-        <v>1417</v>
+        <v>1409</v>
       </c>
       <c r="I233" s="26" t="s">
-        <v>1415</v>
+        <v>1407</v>
       </c>
       <c r="J233" s="23"/>
       <c r="K233" s="18"/>
@@ -22831,18 +22819,10 @@
       </c>
       <c r="H234" s="5"/>
       <c r="I234" s="5"/>
-      <c r="J234" s="22" t="s">
-        <v>1244</v>
-      </c>
-      <c r="K234" s="22" t="s">
-        <v>1243</v>
-      </c>
-      <c r="L234" s="22" t="s">
-        <v>1242</v>
-      </c>
-      <c r="M234" s="22" t="s">
-        <v>1241</v>
-      </c>
+      <c r="J234" s="36"/>
+      <c r="K234" s="36"/>
+      <c r="L234" s="36"/>
+      <c r="M234" s="36"/>
     </row>
     <row r="235" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A235" s="2" t="s">
@@ -22869,18 +22849,10 @@
       </c>
       <c r="H235" s="2"/>
       <c r="I235" s="2"/>
-      <c r="J235" s="21" t="s">
-        <v>1401</v>
-      </c>
-      <c r="K235" s="21" t="s">
-        <v>1403</v>
-      </c>
-      <c r="L235" s="21" t="s">
-        <v>1402</v>
-      </c>
-      <c r="M235" s="21" t="s">
-        <v>1400</v>
-      </c>
+      <c r="J235" s="37"/>
+      <c r="K235" s="37"/>
+      <c r="L235" s="37"/>
+      <c r="M235" s="37"/>
     </row>
     <row r="236" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A236" s="5" t="s">
@@ -23722,16 +23694,16 @@
       <c r="H262" s="5"/>
       <c r="I262" s="5"/>
       <c r="J262" s="22" t="s">
-        <v>1276</v>
+        <v>1272</v>
       </c>
       <c r="K262" s="27" t="s">
-        <v>1275</v>
+        <v>1271</v>
       </c>
       <c r="L262" s="22" t="s">
-        <v>1274</v>
+        <v>1270</v>
       </c>
       <c r="M262" s="22" t="s">
-        <v>1273</v>
+        <v>1269</v>
       </c>
     </row>
     <row r="263" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -23926,7 +23898,7 @@
       <c r="H268" s="2"/>
       <c r="I268" s="2"/>
       <c r="J268" s="21" t="s">
-        <v>1310</v>
+        <v>1306</v>
       </c>
       <c r="K268" s="16"/>
       <c r="L268" s="16"/>
@@ -24390,12 +24362,12 @@
       <c r="H283" s="2"/>
       <c r="I283" s="2"/>
       <c r="J283" s="21" t="s">
-        <v>1353</v>
+        <v>1349</v>
       </c>
       <c r="K283" s="16"/>
       <c r="L283" s="16"/>
       <c r="M283" s="21" t="s">
-        <v>1366</v>
+        <v>1362</v>
       </c>
     </row>
     <row r="284" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -24830,16 +24802,16 @@
       <c r="H297" s="2"/>
       <c r="I297" s="2"/>
       <c r="J297" s="21" t="s">
-        <v>1288</v>
+        <v>1284</v>
       </c>
       <c r="K297" s="21" t="s">
-        <v>1289</v>
+        <v>1285</v>
       </c>
       <c r="L297" s="21" t="s">
-        <v>1290</v>
+        <v>1286</v>
       </c>
       <c r="M297" s="21" t="s">
-        <v>1291</v>
+        <v>1287</v>
       </c>
     </row>
     <row r="298" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -24868,16 +24840,16 @@
       <c r="H298" s="5"/>
       <c r="I298" s="5"/>
       <c r="J298" s="22" t="s">
+        <v>1330</v>
+      </c>
+      <c r="K298" s="22" t="s">
+        <v>1332</v>
+      </c>
+      <c r="L298" s="22" t="s">
+        <v>1333</v>
+      </c>
+      <c r="M298" s="22" t="s">
         <v>1334</v>
-      </c>
-      <c r="K298" s="22" t="s">
-        <v>1336</v>
-      </c>
-      <c r="L298" s="22" t="s">
-        <v>1337</v>
-      </c>
-      <c r="M298" s="22" t="s">
-        <v>1338</v>
       </c>
     </row>
     <row r="299" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -25478,10 +25450,10 @@
       <c r="H317" s="2"/>
       <c r="I317" s="2"/>
       <c r="J317" s="21" t="s">
-        <v>1308</v>
+        <v>1304</v>
       </c>
       <c r="K317" s="21" t="s">
-        <v>1309</v>
+        <v>1305</v>
       </c>
       <c r="L317" s="16"/>
       <c r="M317" s="16"/>
@@ -25512,16 +25484,16 @@
       <c r="H318" s="5"/>
       <c r="I318" s="5"/>
       <c r="J318" s="22" t="s">
-        <v>1383</v>
+        <v>1379</v>
       </c>
       <c r="K318" s="22" t="s">
-        <v>1384</v>
+        <v>1380</v>
       </c>
       <c r="L318" s="22" t="s">
-        <v>1385</v>
+        <v>1381</v>
       </c>
       <c r="M318" s="22" t="s">
-        <v>1386</v>
+        <v>1382</v>
       </c>
     </row>
     <row r="319" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -25806,16 +25778,16 @@
       <c r="H327" s="5"/>
       <c r="I327" s="5"/>
       <c r="J327" s="22" t="s">
-        <v>1269</v>
+        <v>1265</v>
       </c>
       <c r="K327" s="22" t="s">
-        <v>1270</v>
+        <v>1266</v>
       </c>
       <c r="L327" s="22" t="s">
-        <v>1271</v>
+        <v>1267</v>
       </c>
       <c r="M327" s="22" t="s">
-        <v>1272</v>
+        <v>1268</v>
       </c>
     </row>
     <row r="328" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -25844,16 +25816,16 @@
       <c r="H328" s="5"/>
       <c r="I328" s="5"/>
       <c r="J328" s="22" t="s">
-        <v>1292</v>
+        <v>1288</v>
       </c>
       <c r="K328" s="22" t="s">
-        <v>1294</v>
+        <v>1290</v>
       </c>
       <c r="L328" s="22" t="s">
-        <v>1295</v>
+        <v>1291</v>
       </c>
       <c r="M328" s="22" t="s">
-        <v>1293</v>
+        <v>1289</v>
       </c>
     </row>
     <row r="329" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -25882,16 +25854,16 @@
       <c r="H329" s="5"/>
       <c r="I329" s="5"/>
       <c r="J329" s="22" t="s">
-        <v>1396</v>
+        <v>1392</v>
       </c>
       <c r="K329" s="22" t="s">
-        <v>1397</v>
+        <v>1393</v>
       </c>
       <c r="L329" s="22" t="s">
-        <v>1398</v>
+        <v>1394</v>
       </c>
       <c r="M329" s="22" t="s">
-        <v>1399</v>
+        <v>1395</v>
       </c>
     </row>
     <row r="330" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -26079,7 +26051,7 @@
         <v>1049</v>
       </c>
       <c r="M335" s="23" t="s">
-        <v>1430</v>
+        <v>1422</v>
       </c>
     </row>
     <row r="336" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -26184,16 +26156,16 @@
       <c r="H338" s="5"/>
       <c r="I338" s="5"/>
       <c r="J338" s="22" t="s">
-        <v>1326</v>
+        <v>1322</v>
       </c>
       <c r="K338" s="22" t="s">
-        <v>1328</v>
+        <v>1324</v>
       </c>
       <c r="L338" s="22" t="s">
-        <v>1329</v>
+        <v>1325</v>
       </c>
       <c r="M338" s="22" t="s">
-        <v>1327</v>
+        <v>1323</v>
       </c>
     </row>
     <row r="339" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -26562,19 +26534,19 @@
       <c r="I351" s="25"/>
     </row>
     <row r="352" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A352" s="33"/>
-      <c r="B352" s="33"/>
-      <c r="C352" s="34"/>
-      <c r="D352" s="34"/>
-      <c r="E352" s="34"/>
-      <c r="F352" s="34"/>
-      <c r="G352" s="34"/>
-      <c r="H352" s="34"/>
-      <c r="I352" s="34"/>
-      <c r="J352" s="34"/>
-      <c r="K352" s="34"/>
-      <c r="L352" s="34"/>
-      <c r="M352" s="34"/>
+      <c r="A352" s="34"/>
+      <c r="B352" s="34"/>
+      <c r="C352" s="35"/>
+      <c r="D352" s="35"/>
+      <c r="E352" s="35"/>
+      <c r="F352" s="35"/>
+      <c r="G352" s="35"/>
+      <c r="H352" s="35"/>
+      <c r="I352" s="35"/>
+      <c r="J352" s="35"/>
+      <c r="K352" s="35"/>
+      <c r="L352" s="35"/>
+      <c r="M352" s="35"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:M350" xr:uid="{00000000-0009-0000-0000-000001000000}">
@@ -26845,187 +26817,179 @@
     <hyperlink ref="L130" r:id="rId257" xr:uid="{25C0EC99-4084-4EEF-8D04-23E9DCB95415}"/>
     <hyperlink ref="K130" r:id="rId258" xr:uid="{C82AC3D4-9CFE-4DA0-A994-F2D832EFBE22}"/>
     <hyperlink ref="M130" r:id="rId259" xr:uid="{8EE95FD2-85B2-4D89-80C3-FE66F6A15996}"/>
-    <hyperlink ref="M234" r:id="rId260" xr:uid="{AE0A8815-AA89-4A5B-8032-A049602C807E}"/>
-    <hyperlink ref="L234" r:id="rId261" xr:uid="{F037A08E-7B3F-4B50-BB9C-CB755168BA57}"/>
-    <hyperlink ref="K234" r:id="rId262" xr:uid="{837CD94E-C3C4-47A7-B684-840E6448562B}"/>
-    <hyperlink ref="J234" r:id="rId263" xr:uid="{992C4E59-CBBB-4B12-929A-5427D18F893E}"/>
-    <hyperlink ref="M108" r:id="rId264" xr:uid="{ED74A614-5EBD-4739-B94F-EB20107FB2D6}"/>
-    <hyperlink ref="K108" r:id="rId265" xr:uid="{C6F59F61-A257-45AF-877F-39BC3306D4EA}"/>
-    <hyperlink ref="J108" r:id="rId266" xr:uid="{7464499A-5BA1-4D8C-A229-42B61D70F2C5}"/>
-    <hyperlink ref="L108" r:id="rId267" xr:uid="{FF331B10-ACB3-4E9D-B260-1C7BB046E4F6}"/>
-    <hyperlink ref="J66" r:id="rId268" xr:uid="{9227A9C3-9E81-43B2-A038-1B69A37A90B8}"/>
-    <hyperlink ref="L66" r:id="rId269" xr:uid="{5A822F7D-B80A-4946-ABEE-846FCD2D1760}"/>
-    <hyperlink ref="K66" r:id="rId270" xr:uid="{0EE2CB08-A09A-4451-B516-966038CF27FD}"/>
-    <hyperlink ref="M66" r:id="rId271" xr:uid="{BE651F56-FABD-41BF-8A50-59B08D48CF9C}"/>
-    <hyperlink ref="J131" r:id="rId272" xr:uid="{D2418C1C-EF4A-4036-8AF3-89D91FDD787B}"/>
-    <hyperlink ref="L131" r:id="rId273" xr:uid="{C99311E7-1188-4AF4-8A2C-D3661410CC6F}"/>
-    <hyperlink ref="K131" r:id="rId274" xr:uid="{E522DBF5-F59E-4635-B411-BBFEC0FFD3CB}"/>
-    <hyperlink ref="M131" r:id="rId275" xr:uid="{A7083C05-0F97-4C39-ADE9-A068F47B6F9C}"/>
-    <hyperlink ref="J67" r:id="rId276" xr:uid="{30BEDCE5-C818-49EA-8DC0-3FA7851BC49D}"/>
-    <hyperlink ref="L67" r:id="rId277" xr:uid="{C05CACFF-DC02-4C34-8C7D-D154B5D2EC99}"/>
-    <hyperlink ref="K67" r:id="rId278" xr:uid="{9CD9860A-9DDE-4A80-A43E-CC3BEA61881E}"/>
-    <hyperlink ref="M67" r:id="rId279" xr:uid="{4B66A3B2-9EED-4A1E-B926-B8025B5799C3}"/>
-    <hyperlink ref="J167" r:id="rId280" xr:uid="{04D82AC4-9373-4495-B029-1B0E35B56C71}"/>
-    <hyperlink ref="K167" r:id="rId281" xr:uid="{9DE0D6F8-DAC5-43DA-B52E-4E4494B7C5F6}"/>
-    <hyperlink ref="L167" r:id="rId282" xr:uid="{E9AF79E0-2AA2-4687-BEFE-0F7ED15059AE}"/>
-    <hyperlink ref="M167" r:id="rId283" xr:uid="{90FA869D-615C-4490-9D54-21A639C95D57}"/>
-    <hyperlink ref="J3" r:id="rId284" xr:uid="{186189FC-B189-48B5-9141-CCF3794EB2B3}"/>
-    <hyperlink ref="K3" r:id="rId285" xr:uid="{7A34B5FE-017C-4B67-BBA7-3D01A773A960}"/>
-    <hyperlink ref="M3" r:id="rId286" xr:uid="{89B1D8F3-87FA-4554-BA8E-5ABFFA8FE0DB}"/>
-    <hyperlink ref="J327" r:id="rId287" xr:uid="{8E5153DE-9C00-4689-9D84-6F1CC94C83C8}"/>
-    <hyperlink ref="K327" r:id="rId288" xr:uid="{1C6295FC-CBEE-4117-B836-EB66FABBF5F8}"/>
-    <hyperlink ref="L327" r:id="rId289" xr:uid="{973BFCFF-5877-4D0C-B83E-51120FFF284B}"/>
-    <hyperlink ref="M327" r:id="rId290" xr:uid="{2EE8AFEC-9394-4014-90EF-EFCBC4F87F67}"/>
-    <hyperlink ref="L262" r:id="rId291" xr:uid="{EA571617-EAAF-4298-A444-1686ADD1D3D5}"/>
-    <hyperlink ref="K262" r:id="rId292" xr:uid="{AC84840B-F3D1-480B-BB39-024179B2F2FE}"/>
-    <hyperlink ref="J262" r:id="rId293" xr:uid="{E8B9E159-E076-416B-B54D-E3B95F01ED75}"/>
-    <hyperlink ref="J132" r:id="rId294" xr:uid="{B450D7E7-5FFA-413C-8E43-1B6EB18697DE}"/>
-    <hyperlink ref="K132" r:id="rId295" xr:uid="{33DA5BD8-3FDC-4BEE-AD0F-56CC1D26927A}"/>
-    <hyperlink ref="L132" r:id="rId296" xr:uid="{692DD2B8-162E-41D4-B102-9E744EBF34FC}"/>
-    <hyperlink ref="M132" r:id="rId297" xr:uid="{374B1D5B-6330-4DD9-AC3A-273CC12CB3CA}"/>
-    <hyperlink ref="J151" r:id="rId298" xr:uid="{461E7030-4225-4F51-830A-F0A914765891}"/>
-    <hyperlink ref="K151" r:id="rId299" xr:uid="{63D4F047-34D7-4DB3-A863-D338E082518F}"/>
-    <hyperlink ref="L151" r:id="rId300" xr:uid="{3E2E93AE-B986-4030-A5A4-DCF3E38CCAFC}"/>
-    <hyperlink ref="M151" r:id="rId301" xr:uid="{89DBB7D9-B012-4778-86BA-B88448122C6F}"/>
-    <hyperlink ref="K79" r:id="rId302" xr:uid="{1CC3B30D-55E3-48C4-958E-2194300E7D16}"/>
-    <hyperlink ref="M79" r:id="rId303" xr:uid="{250A8EE6-9C28-4FB2-9D35-73B8CC2B4E00}"/>
-    <hyperlink ref="M262" r:id="rId304" xr:uid="{09E505D1-5E14-4B56-9CB8-B521B3B81A60}"/>
-    <hyperlink ref="L79" r:id="rId305" xr:uid="{A98CD08F-B3A3-4243-AC18-4D36F4536165}"/>
-    <hyperlink ref="J297" r:id="rId306" xr:uid="{6D66CEBB-CAFA-43E6-AE15-E5FD81162B6E}"/>
-    <hyperlink ref="K297" r:id="rId307" xr:uid="{6F7C2771-FFE8-4F6A-9417-3F9278D90766}"/>
-    <hyperlink ref="L297" r:id="rId308" xr:uid="{1FEE7F89-264D-46C0-90B0-BE6603006F15}"/>
-    <hyperlink ref="M297" r:id="rId309" xr:uid="{13258245-AED3-4740-868D-25D308564107}"/>
-    <hyperlink ref="J328" r:id="rId310" xr:uid="{C25F4DDE-DEF0-48B2-B142-958599703B6B}"/>
-    <hyperlink ref="M328" r:id="rId311" xr:uid="{64D94DEC-FDCB-4B47-8ED0-CFAE81F35579}"/>
-    <hyperlink ref="K328" r:id="rId312" xr:uid="{74EF847F-3849-4C10-A31E-2A821F251DC3}"/>
-    <hyperlink ref="L328" r:id="rId313" xr:uid="{43E6FB73-BFB5-4757-BB0D-7665CD644538}"/>
-    <hyperlink ref="M98" r:id="rId314" xr:uid="{995E09AF-C1E8-46E9-A2F2-E51BB4C8802E}"/>
-    <hyperlink ref="J41" r:id="rId315" xr:uid="{84B8E2A8-8EF7-47F0-9A21-ABC7086C904B}"/>
-    <hyperlink ref="M152" r:id="rId316" xr:uid="{7355F602-54A8-4514-A6D3-E00D8F73A9EC}"/>
-    <hyperlink ref="K152" r:id="rId317" xr:uid="{AA64C7A4-22C4-4714-8118-7E4E11736E0D}"/>
-    <hyperlink ref="J152" r:id="rId318" xr:uid="{66D5E096-C1AA-4813-8367-8813F33D8F7B}"/>
-    <hyperlink ref="L152" r:id="rId319" xr:uid="{088F396F-DDB0-4E9C-9EFA-93CF44B5CF21}"/>
-    <hyperlink ref="J209" r:id="rId320" xr:uid="{A476BAFF-FC7D-4364-8C47-B546C0FAEE1A}"/>
-    <hyperlink ref="K209" r:id="rId321" xr:uid="{121D0C05-91A0-40FA-81D2-DE84701C9D4A}"/>
-    <hyperlink ref="L209" r:id="rId322" xr:uid="{74F955A8-D058-4F2F-B305-775CAF52E311}"/>
-    <hyperlink ref="M209" r:id="rId323" xr:uid="{12F46A80-0F27-4F05-BF49-AF24094366CF}"/>
-    <hyperlink ref="M199" r:id="rId324" xr:uid="{8E864CFD-E74B-4019-A2B2-4706CA2FD461}"/>
-    <hyperlink ref="J199" r:id="rId325" xr:uid="{31A2FFC9-8611-4C66-85B2-A520F1E268C4}"/>
-    <hyperlink ref="J317" r:id="rId326" xr:uid="{AB3A3661-592C-48A5-ACE8-7849626E100E}"/>
-    <hyperlink ref="K317" r:id="rId327" xr:uid="{DC19933C-125E-400C-9DFC-4F8D6B24C97A}"/>
-    <hyperlink ref="J268" r:id="rId328" xr:uid="{6562872A-C53C-4F7A-B801-BC40C4E3CCC1}"/>
-    <hyperlink ref="J119" r:id="rId329" xr:uid="{5B13E2CD-8364-4740-AD00-ABF4FC0A8692}"/>
-    <hyperlink ref="K119" r:id="rId330" xr:uid="{F1FE7A53-8846-4620-A384-64E6E1C19E55}"/>
-    <hyperlink ref="L119" r:id="rId331" xr:uid="{554794B1-A8F7-4E9E-A0AC-42EC086AA2E4}"/>
-    <hyperlink ref="M119" r:id="rId332" xr:uid="{1A116AA9-0ADA-49AD-A794-14AE8D3FE151}"/>
-    <hyperlink ref="J29" r:id="rId333" xr:uid="{D5A43CA5-B9F3-432D-B2F9-44FC4B3DBD58}"/>
-    <hyperlink ref="K29" r:id="rId334" xr:uid="{930817CD-7C90-4C39-B5F4-1E1F9697BCB5}"/>
-    <hyperlink ref="L29" r:id="rId335" xr:uid="{1CFF83CE-EE93-4C21-9EA7-63E5FCC2F519}"/>
-    <hyperlink ref="M29" r:id="rId336" xr:uid="{18CBF1E8-22B2-4E10-A90D-39AA32EA2C8B}"/>
-    <hyperlink ref="J153" r:id="rId337" xr:uid="{AF53763A-27C2-496A-A7C6-EFB2EAAF55E0}"/>
-    <hyperlink ref="K153" r:id="rId338" xr:uid="{6B170007-30E6-41E1-B8CB-95BDA29DDB2B}"/>
-    <hyperlink ref="L153" r:id="rId339" xr:uid="{7EC3496E-2E1B-4B5D-9FEA-5F2B8AEE7B88}"/>
-    <hyperlink ref="M153" r:id="rId340" xr:uid="{F3A099FF-1F51-4154-9354-D85DE020ED13}"/>
-    <hyperlink ref="J137" r:id="rId341" xr:uid="{33113C3E-D96E-435E-AE16-39788B2C1DE7}"/>
-    <hyperlink ref="M137" r:id="rId342" xr:uid="{73B1B857-6530-40D8-8875-6FCBA7D480BC}"/>
-    <hyperlink ref="J338" r:id="rId343" xr:uid="{136B2C93-7250-4C1B-93C0-3C28345DA9D4}"/>
-    <hyperlink ref="M338" r:id="rId344" xr:uid="{46E8AF26-C80F-43B5-BCD9-1DA8FAF40F3B}"/>
-    <hyperlink ref="K338" r:id="rId345" xr:uid="{6EF79CD8-8AF4-4A4D-8D3F-F3BD88E29EE1}"/>
-    <hyperlink ref="L338" r:id="rId346" xr:uid="{DE6E9178-A430-4395-9E7A-540F30BD3DD5}"/>
-    <hyperlink ref="J219" r:id="rId347" xr:uid="{A886421C-9FA0-4D1D-A555-D75C6BBEC56D}"/>
-    <hyperlink ref="K219" r:id="rId348" xr:uid="{03D0F959-65F0-4576-B1C1-EB2A63DAFFFE}"/>
-    <hyperlink ref="L219" r:id="rId349" xr:uid="{83B6EE5F-0FA0-464A-A871-35882B674CD7}"/>
-    <hyperlink ref="M219" r:id="rId350" xr:uid="{20D12798-4F2D-45D8-B3D9-EEDAC8BA81AA}"/>
-    <hyperlink ref="J298" r:id="rId351" xr:uid="{F5527F66-B3DA-41D8-9765-4CA7EEDC97F1}"/>
-    <hyperlink ref="K298" r:id="rId352" xr:uid="{1A2A15F4-5117-42C7-8B70-CA4AB5970A53}"/>
-    <hyperlink ref="L298" r:id="rId353" xr:uid="{9AB03DF6-2293-4BBA-B95F-D4513057928C}"/>
-    <hyperlink ref="M298" r:id="rId354" xr:uid="{A2E339C5-2DF9-4719-964F-F251CB520C94}"/>
-    <hyperlink ref="K61" r:id="rId355" xr:uid="{377B7786-3EAF-416F-99C6-8C77872E4C23}"/>
-    <hyperlink ref="J61" r:id="rId356" xr:uid="{0854386D-6229-4879-9457-DDA376455E76}"/>
-    <hyperlink ref="L61" r:id="rId357" xr:uid="{23628636-C0DC-445A-83E0-3745B69B9189}"/>
-    <hyperlink ref="J200" r:id="rId358" xr:uid="{D0E98960-CCCC-4BE2-BC70-EBA21D7DD8B4}"/>
-    <hyperlink ref="M200" r:id="rId359" xr:uid="{D49963B7-E86C-4490-977A-501B8A78A3DD}"/>
-    <hyperlink ref="J229" r:id="rId360" xr:uid="{87D0FA26-A909-45F1-BD49-F86D89AF1A58}"/>
-    <hyperlink ref="L229" r:id="rId361" xr:uid="{A838D8C4-AC0D-46CD-BEB4-4D5804C43945}"/>
-    <hyperlink ref="K229" r:id="rId362" xr:uid="{D9C5DFF7-9BF6-4BF2-83DC-F549252E49F2}"/>
-    <hyperlink ref="M229" r:id="rId363" xr:uid="{9D3DAEF5-BF30-4D21-916D-450F5C49DEF0}"/>
-    <hyperlink ref="M201" r:id="rId364" xr:uid="{9F7C5EF6-018D-483C-B59B-3DE77ACC60D5}"/>
-    <hyperlink ref="K201" r:id="rId365" xr:uid="{0482AEA3-29E3-4285-BA7C-61171C0896C9}"/>
-    <hyperlink ref="L201" r:id="rId366" xr:uid="{D015EE26-7E89-4DC7-8E92-938B53864255}"/>
-    <hyperlink ref="J201" r:id="rId367" xr:uid="{F3B3A811-947E-4A64-9FD3-9D295407E06F}"/>
-    <hyperlink ref="J141" r:id="rId368" xr:uid="{59736F95-E649-4CFA-8A45-53EF3C5F5FE6}"/>
-    <hyperlink ref="K141" r:id="rId369" xr:uid="{ED28EC78-A0B8-4996-B314-2E390CDDA886}"/>
-    <hyperlink ref="L141" r:id="rId370" xr:uid="{13FC8DC5-72F5-4379-BE4E-9923F5114396}"/>
-    <hyperlink ref="M141" r:id="rId371" xr:uid="{4DB2DF46-3D91-485F-86D1-A018F3AA4C0B}"/>
-    <hyperlink ref="J179" r:id="rId372" xr:uid="{264B41A9-B5FA-48AF-ACB2-AAE3C399AE90}"/>
-    <hyperlink ref="K179" r:id="rId373" xr:uid="{61EE2789-FED2-43B9-A813-328A352754CA}"/>
-    <hyperlink ref="L179" r:id="rId374" xr:uid="{728AEF58-6A7C-4829-A776-9E1F1A2FEC31}"/>
-    <hyperlink ref="M179" r:id="rId375" xr:uid="{1919B1A3-793A-4D63-B5AE-8E4498DDC235}"/>
-    <hyperlink ref="J120" r:id="rId376" xr:uid="{9EED662A-9B0A-42E9-886E-56A9B743EA4A}"/>
-    <hyperlink ref="K120" r:id="rId377" xr:uid="{4EF1B325-BE49-4D6E-9CBD-27713228D023}"/>
-    <hyperlink ref="L120" r:id="rId378" xr:uid="{79D2603C-C10F-4869-8AFD-73E90DC5158A}"/>
-    <hyperlink ref="M120" r:id="rId379" xr:uid="{07C54EF0-2A81-4580-841B-48FE8C5BE427}"/>
-    <hyperlink ref="J202" r:id="rId380" xr:uid="{240A6E84-68A0-4B87-82E1-562572ED7AB7}"/>
-    <hyperlink ref="L202" r:id="rId381" xr:uid="{7BD4B96C-8B86-4D4B-9D11-A81A1AFC1913}"/>
-    <hyperlink ref="M202" r:id="rId382" xr:uid="{69B03112-4BCA-44CA-8AB4-995FF08CC991}"/>
-    <hyperlink ref="J283" r:id="rId383" xr:uid="{3EABF4BD-FDFB-4024-BB99-D5FB80F7420C}"/>
-    <hyperlink ref="M283" r:id="rId384" xr:uid="{8E10395F-6237-4A45-9FAE-9547ED9F3FDB}"/>
-    <hyperlink ref="J203" r:id="rId385" xr:uid="{2FB5AD72-AE18-411D-913F-8A9E4798293B}"/>
-    <hyperlink ref="K203" r:id="rId386" xr:uid="{40BC0523-4BBD-4DC5-8035-5B2FA54C84DD}"/>
-    <hyperlink ref="L203" r:id="rId387" xr:uid="{C103903A-DBC4-4FDD-B63A-AAF14138F219}"/>
-    <hyperlink ref="M203" r:id="rId388" xr:uid="{88D8FF20-9A07-4692-9DA6-7E9441D8853A}"/>
-    <hyperlink ref="J121" r:id="rId389" xr:uid="{CDF21456-7EE7-4FAF-9E29-AC3095E8B710}"/>
-    <hyperlink ref="K121" r:id="rId390" xr:uid="{FB72FBED-F0D8-4EEB-8609-DC41E244C6D5}"/>
-    <hyperlink ref="L121" r:id="rId391" xr:uid="{9FE6BB21-D205-4F42-A4A1-04B7B3B8B867}"/>
-    <hyperlink ref="M121" r:id="rId392" xr:uid="{B259A195-3609-4A06-AC4B-74DA482DE1A8}"/>
-    <hyperlink ref="J180" r:id="rId393" xr:uid="{C432A164-9BBF-401D-A2D8-8A71573C54D8}"/>
-    <hyperlink ref="K180" r:id="rId394" xr:uid="{2D2E3A14-600E-4CFD-8A4E-F0B61820295E}"/>
-    <hyperlink ref="L180" r:id="rId395" xr:uid="{0E159A7A-119E-44FF-A05B-0FFDC2D4E34A}"/>
-    <hyperlink ref="M180" r:id="rId396" xr:uid="{29D68BF5-F2DB-409B-99A9-0CE74D783774}"/>
-    <hyperlink ref="M15" r:id="rId397" xr:uid="{26DC8B78-F5FC-4FFE-9BEB-C68A3D718BF5}"/>
-    <hyperlink ref="J15" r:id="rId398" xr:uid="{36999AC1-13FC-4C81-A5FE-1AE970997895}"/>
-    <hyperlink ref="K15" r:id="rId399" xr:uid="{F1B6CDB3-D7DB-4041-8DA1-36CF172DB220}"/>
-    <hyperlink ref="L15" r:id="rId400" xr:uid="{36074799-65FC-4632-AA92-F02DCCB993A5}"/>
-    <hyperlink ref="J318" r:id="rId401" xr:uid="{7B1640BB-82E7-44A9-BD5B-6FD8C51CC5C4}"/>
-    <hyperlink ref="K318" r:id="rId402" xr:uid="{1BEDE21F-61F4-4AA1-A729-C684C7C4A9A7}"/>
-    <hyperlink ref="L318" r:id="rId403" xr:uid="{626BDFDE-7AC6-43CF-85E2-7D50E0B1B4EC}"/>
-    <hyperlink ref="M318" r:id="rId404" xr:uid="{99EBF6F1-06EB-4315-A3AE-AB9957D3FB2B}"/>
-    <hyperlink ref="M47" r:id="rId405" xr:uid="{7B07B612-3A88-4B60-886F-6FC970BB6B41}"/>
-    <hyperlink ref="J99" r:id="rId406" xr:uid="{0D0C9636-A1BE-4572-9F60-17DA53A1D9B8}"/>
-    <hyperlink ref="K99" r:id="rId407" xr:uid="{73689F04-7E3B-430A-988E-472883578A46}"/>
-    <hyperlink ref="M99" r:id="rId408" xr:uid="{9410E670-EECB-417E-9A31-D3949A0214B2}"/>
-    <hyperlink ref="L99" r:id="rId409" xr:uid="{A215DA8C-109A-4819-9C6D-80C0A1492AC1}"/>
-    <hyperlink ref="J154" r:id="rId410" xr:uid="{8507B41C-7E70-400C-930C-AB114BA6509E}"/>
-    <hyperlink ref="K154" r:id="rId411" xr:uid="{E9FE295A-2D43-420A-8A9E-10F016D11B6C}"/>
-    <hyperlink ref="L154" r:id="rId412" xr:uid="{BE50457E-5FF4-46CE-983A-8A1E71BB846E}"/>
-    <hyperlink ref="M154" r:id="rId413" xr:uid="{5217E048-4675-43D9-9163-562318C43A55}"/>
-    <hyperlink ref="J329" r:id="rId414" xr:uid="{904205CF-7EB6-4895-AFCD-F3B24BB02260}"/>
-    <hyperlink ref="K329" r:id="rId415" xr:uid="{2C2AE4C7-0238-4B56-89D6-B1E30FE2A47E}"/>
-    <hyperlink ref="L329" r:id="rId416" xr:uid="{5F95A1EF-F351-4326-B4B0-0BE11CC3FD81}"/>
-    <hyperlink ref="M329" r:id="rId417" xr:uid="{88820289-C3F9-4DB3-926D-95F74FA46E7F}"/>
-    <hyperlink ref="M235" r:id="rId418" xr:uid="{84013A51-65D7-4364-80AD-68AB09966D22}"/>
-    <hyperlink ref="J235" r:id="rId419" xr:uid="{666D654D-08F1-4058-B107-A245896B6FC1}"/>
-    <hyperlink ref="L235" r:id="rId420" xr:uid="{0E8A8878-07DA-42EE-9834-EEE7B9753309}"/>
-    <hyperlink ref="K235" r:id="rId421" xr:uid="{14603315-4B99-4DF1-9E49-DB6FE13D0C09}"/>
-    <hyperlink ref="J181" r:id="rId422" xr:uid="{0DE0D3CC-91C4-48C1-A2B4-EC846B5D1082}"/>
-    <hyperlink ref="K181" r:id="rId423" xr:uid="{B17BCE6D-1CA5-4D3F-9CB9-D26C8358CF7F}"/>
-    <hyperlink ref="L181" r:id="rId424" xr:uid="{ECBAD3DE-BD62-4A89-A694-011DE2D981C1}"/>
-    <hyperlink ref="M181" r:id="rId425" xr:uid="{FDDAB7EC-3DDF-4C42-B006-1E9755E3C809}"/>
-    <hyperlink ref="J68" r:id="rId426" xr:uid="{462837B2-0B52-489B-95BC-8BA6183CC41A}"/>
-    <hyperlink ref="M68" r:id="rId427" xr:uid="{F42FD553-6EB7-4B88-A9FE-261718A340E8}"/>
-    <hyperlink ref="K68" r:id="rId428" xr:uid="{7A183CAD-5D6A-4E1E-A490-A2287DC0528C}"/>
-    <hyperlink ref="L68" r:id="rId429" xr:uid="{B22A6BB4-2BF6-435B-A883-4962FAAAEE8F}"/>
-    <hyperlink ref="J69" r:id="rId430" xr:uid="{F30B54DC-2EEE-4B78-93F0-7E62616FB4DC}"/>
-    <hyperlink ref="M69" r:id="rId431" xr:uid="{B5B739A5-B17C-40F7-8205-0AA4763BC714}"/>
-    <hyperlink ref="I233" r:id="rId432" xr:uid="{C3369525-B7A0-4412-8D59-0C493A78E1DC}"/>
-    <hyperlink ref="J62" r:id="rId433" xr:uid="{E7329603-2EDD-44F0-B789-E1D85A13A5AF}"/>
-    <hyperlink ref="M62" r:id="rId434" xr:uid="{2A04F1A5-411E-4112-96AF-11194F0F7BB9}"/>
-    <hyperlink ref="K62" r:id="rId435" xr:uid="{0386DF53-8D0D-44E0-8911-4355A04799F9}"/>
-    <hyperlink ref="L62" r:id="rId436" xr:uid="{8C766B81-71F9-4A3D-A568-5595B2174541}"/>
-    <hyperlink ref="J98" r:id="rId437" xr:uid="{CF0A4B26-01DE-4363-8D0A-7FDDD09CFCDE}"/>
-    <hyperlink ref="L98" r:id="rId438" xr:uid="{CD04CC97-53AD-43B1-ABAA-2D4FE039CB55}"/>
-    <hyperlink ref="K98" r:id="rId439" xr:uid="{094EBB15-996A-4155-B60F-1048DF22330D}"/>
-    <hyperlink ref="M41" r:id="rId440" xr:uid="{E18AE4E3-ACC6-4772-AF56-2A6606909541}"/>
+    <hyperlink ref="M108" r:id="rId260" xr:uid="{ED74A614-5EBD-4739-B94F-EB20107FB2D6}"/>
+    <hyperlink ref="K108" r:id="rId261" xr:uid="{C6F59F61-A257-45AF-877F-39BC3306D4EA}"/>
+    <hyperlink ref="J108" r:id="rId262" xr:uid="{7464499A-5BA1-4D8C-A229-42B61D70F2C5}"/>
+    <hyperlink ref="L108" r:id="rId263" xr:uid="{FF331B10-ACB3-4E9D-B260-1C7BB046E4F6}"/>
+    <hyperlink ref="J66" r:id="rId264" xr:uid="{9227A9C3-9E81-43B2-A038-1B69A37A90B8}"/>
+    <hyperlink ref="L66" r:id="rId265" xr:uid="{5A822F7D-B80A-4946-ABEE-846FCD2D1760}"/>
+    <hyperlink ref="K66" r:id="rId266" xr:uid="{0EE2CB08-A09A-4451-B516-966038CF27FD}"/>
+    <hyperlink ref="M66" r:id="rId267" xr:uid="{BE651F56-FABD-41BF-8A50-59B08D48CF9C}"/>
+    <hyperlink ref="J131" r:id="rId268" xr:uid="{D2418C1C-EF4A-4036-8AF3-89D91FDD787B}"/>
+    <hyperlink ref="L131" r:id="rId269" xr:uid="{C99311E7-1188-4AF4-8A2C-D3661410CC6F}"/>
+    <hyperlink ref="K131" r:id="rId270" xr:uid="{E522DBF5-F59E-4635-B411-BBFEC0FFD3CB}"/>
+    <hyperlink ref="M131" r:id="rId271" xr:uid="{A7083C05-0F97-4C39-ADE9-A068F47B6F9C}"/>
+    <hyperlink ref="J67" r:id="rId272" xr:uid="{30BEDCE5-C818-49EA-8DC0-3FA7851BC49D}"/>
+    <hyperlink ref="L67" r:id="rId273" xr:uid="{C05CACFF-DC02-4C34-8C7D-D154B5D2EC99}"/>
+    <hyperlink ref="K67" r:id="rId274" xr:uid="{9CD9860A-9DDE-4A80-A43E-CC3BEA61881E}"/>
+    <hyperlink ref="M67" r:id="rId275" xr:uid="{4B66A3B2-9EED-4A1E-B926-B8025B5799C3}"/>
+    <hyperlink ref="J167" r:id="rId276" xr:uid="{04D82AC4-9373-4495-B029-1B0E35B56C71}"/>
+    <hyperlink ref="K167" r:id="rId277" xr:uid="{9DE0D6F8-DAC5-43DA-B52E-4E4494B7C5F6}"/>
+    <hyperlink ref="L167" r:id="rId278" xr:uid="{E9AF79E0-2AA2-4687-BEFE-0F7ED15059AE}"/>
+    <hyperlink ref="M167" r:id="rId279" xr:uid="{90FA869D-615C-4490-9D54-21A639C95D57}"/>
+    <hyperlink ref="J3" r:id="rId280" xr:uid="{186189FC-B189-48B5-9141-CCF3794EB2B3}"/>
+    <hyperlink ref="K3" r:id="rId281" xr:uid="{7A34B5FE-017C-4B67-BBA7-3D01A773A960}"/>
+    <hyperlink ref="M3" r:id="rId282" xr:uid="{89B1D8F3-87FA-4554-BA8E-5ABFFA8FE0DB}"/>
+    <hyperlink ref="J327" r:id="rId283" xr:uid="{8E5153DE-9C00-4689-9D84-6F1CC94C83C8}"/>
+    <hyperlink ref="K327" r:id="rId284" xr:uid="{1C6295FC-CBEE-4117-B836-EB66FABBF5F8}"/>
+    <hyperlink ref="L327" r:id="rId285" xr:uid="{973BFCFF-5877-4D0C-B83E-51120FFF284B}"/>
+    <hyperlink ref="M327" r:id="rId286" xr:uid="{2EE8AFEC-9394-4014-90EF-EFCBC4F87F67}"/>
+    <hyperlink ref="L262" r:id="rId287" xr:uid="{EA571617-EAAF-4298-A444-1686ADD1D3D5}"/>
+    <hyperlink ref="K262" r:id="rId288" xr:uid="{AC84840B-F3D1-480B-BB39-024179B2F2FE}"/>
+    <hyperlink ref="J262" r:id="rId289" xr:uid="{E8B9E159-E076-416B-B54D-E3B95F01ED75}"/>
+    <hyperlink ref="J132" r:id="rId290" xr:uid="{B450D7E7-5FFA-413C-8E43-1B6EB18697DE}"/>
+    <hyperlink ref="K132" r:id="rId291" xr:uid="{33DA5BD8-3FDC-4BEE-AD0F-56CC1D26927A}"/>
+    <hyperlink ref="L132" r:id="rId292" xr:uid="{692DD2B8-162E-41D4-B102-9E744EBF34FC}"/>
+    <hyperlink ref="M132" r:id="rId293" xr:uid="{374B1D5B-6330-4DD9-AC3A-273CC12CB3CA}"/>
+    <hyperlink ref="J151" r:id="rId294" xr:uid="{461E7030-4225-4F51-830A-F0A914765891}"/>
+    <hyperlink ref="K151" r:id="rId295" xr:uid="{63D4F047-34D7-4DB3-A863-D338E082518F}"/>
+    <hyperlink ref="L151" r:id="rId296" xr:uid="{3E2E93AE-B986-4030-A5A4-DCF3E38CCAFC}"/>
+    <hyperlink ref="M151" r:id="rId297" xr:uid="{89DBB7D9-B012-4778-86BA-B88448122C6F}"/>
+    <hyperlink ref="K79" r:id="rId298" xr:uid="{1CC3B30D-55E3-48C4-958E-2194300E7D16}"/>
+    <hyperlink ref="M79" r:id="rId299" xr:uid="{250A8EE6-9C28-4FB2-9D35-73B8CC2B4E00}"/>
+    <hyperlink ref="M262" r:id="rId300" xr:uid="{09E505D1-5E14-4B56-9CB8-B521B3B81A60}"/>
+    <hyperlink ref="L79" r:id="rId301" xr:uid="{A98CD08F-B3A3-4243-AC18-4D36F4536165}"/>
+    <hyperlink ref="J297" r:id="rId302" xr:uid="{6D66CEBB-CAFA-43E6-AE15-E5FD81162B6E}"/>
+    <hyperlink ref="K297" r:id="rId303" xr:uid="{6F7C2771-FFE8-4F6A-9417-3F9278D90766}"/>
+    <hyperlink ref="L297" r:id="rId304" xr:uid="{1FEE7F89-264D-46C0-90B0-BE6603006F15}"/>
+    <hyperlink ref="M297" r:id="rId305" xr:uid="{13258245-AED3-4740-868D-25D308564107}"/>
+    <hyperlink ref="J328" r:id="rId306" xr:uid="{C25F4DDE-DEF0-48B2-B142-958599703B6B}"/>
+    <hyperlink ref="M328" r:id="rId307" xr:uid="{64D94DEC-FDCB-4B47-8ED0-CFAE81F35579}"/>
+    <hyperlink ref="K328" r:id="rId308" xr:uid="{74EF847F-3849-4C10-A31E-2A821F251DC3}"/>
+    <hyperlink ref="L328" r:id="rId309" xr:uid="{43E6FB73-BFB5-4757-BB0D-7665CD644538}"/>
+    <hyperlink ref="M98" r:id="rId310" xr:uid="{995E09AF-C1E8-46E9-A2F2-E51BB4C8802E}"/>
+    <hyperlink ref="J41" r:id="rId311" xr:uid="{84B8E2A8-8EF7-47F0-9A21-ABC7086C904B}"/>
+    <hyperlink ref="M152" r:id="rId312" xr:uid="{7355F602-54A8-4514-A6D3-E00D8F73A9EC}"/>
+    <hyperlink ref="K152" r:id="rId313" xr:uid="{AA64C7A4-22C4-4714-8118-7E4E11736E0D}"/>
+    <hyperlink ref="J152" r:id="rId314" xr:uid="{66D5E096-C1AA-4813-8367-8813F33D8F7B}"/>
+    <hyperlink ref="L152" r:id="rId315" xr:uid="{088F396F-DDB0-4E9C-9EFA-93CF44B5CF21}"/>
+    <hyperlink ref="J209" r:id="rId316" xr:uid="{A476BAFF-FC7D-4364-8C47-B546C0FAEE1A}"/>
+    <hyperlink ref="K209" r:id="rId317" xr:uid="{121D0C05-91A0-40FA-81D2-DE84701C9D4A}"/>
+    <hyperlink ref="L209" r:id="rId318" xr:uid="{74F955A8-D058-4F2F-B305-775CAF52E311}"/>
+    <hyperlink ref="M209" r:id="rId319" xr:uid="{12F46A80-0F27-4F05-BF49-AF24094366CF}"/>
+    <hyperlink ref="M199" r:id="rId320" xr:uid="{8E864CFD-E74B-4019-A2B2-4706CA2FD461}"/>
+    <hyperlink ref="J199" r:id="rId321" xr:uid="{31A2FFC9-8611-4C66-85B2-A520F1E268C4}"/>
+    <hyperlink ref="J317" r:id="rId322" xr:uid="{AB3A3661-592C-48A5-ACE8-7849626E100E}"/>
+    <hyperlink ref="K317" r:id="rId323" xr:uid="{DC19933C-125E-400C-9DFC-4F8D6B24C97A}"/>
+    <hyperlink ref="J268" r:id="rId324" xr:uid="{6562872A-C53C-4F7A-B801-BC40C4E3CCC1}"/>
+    <hyperlink ref="J119" r:id="rId325" xr:uid="{5B13E2CD-8364-4740-AD00-ABF4FC0A8692}"/>
+    <hyperlink ref="K119" r:id="rId326" xr:uid="{F1FE7A53-8846-4620-A384-64E6E1C19E55}"/>
+    <hyperlink ref="L119" r:id="rId327" xr:uid="{554794B1-A8F7-4E9E-A0AC-42EC086AA2E4}"/>
+    <hyperlink ref="M119" r:id="rId328" xr:uid="{1A116AA9-0ADA-49AD-A794-14AE8D3FE151}"/>
+    <hyperlink ref="J29" r:id="rId329" xr:uid="{D5A43CA5-B9F3-432D-B2F9-44FC4B3DBD58}"/>
+    <hyperlink ref="K29" r:id="rId330" xr:uid="{930817CD-7C90-4C39-B5F4-1E1F9697BCB5}"/>
+    <hyperlink ref="L29" r:id="rId331" xr:uid="{1CFF83CE-EE93-4C21-9EA7-63E5FCC2F519}"/>
+    <hyperlink ref="M29" r:id="rId332" xr:uid="{18CBF1E8-22B2-4E10-A90D-39AA32EA2C8B}"/>
+    <hyperlink ref="J153" r:id="rId333" xr:uid="{AF53763A-27C2-496A-A7C6-EFB2EAAF55E0}"/>
+    <hyperlink ref="K153" r:id="rId334" xr:uid="{6B170007-30E6-41E1-B8CB-95BDA29DDB2B}"/>
+    <hyperlink ref="L153" r:id="rId335" xr:uid="{7EC3496E-2E1B-4B5D-9FEA-5F2B8AEE7B88}"/>
+    <hyperlink ref="M153" r:id="rId336" xr:uid="{F3A099FF-1F51-4154-9354-D85DE020ED13}"/>
+    <hyperlink ref="J137" r:id="rId337" xr:uid="{33113C3E-D96E-435E-AE16-39788B2C1DE7}"/>
+    <hyperlink ref="M137" r:id="rId338" xr:uid="{73B1B857-6530-40D8-8875-6FCBA7D480BC}"/>
+    <hyperlink ref="J338" r:id="rId339" xr:uid="{136B2C93-7250-4C1B-93C0-3C28345DA9D4}"/>
+    <hyperlink ref="M338" r:id="rId340" xr:uid="{46E8AF26-C80F-43B5-BCD9-1DA8FAF40F3B}"/>
+    <hyperlink ref="K338" r:id="rId341" xr:uid="{6EF79CD8-8AF4-4A4D-8D3F-F3BD88E29EE1}"/>
+    <hyperlink ref="L338" r:id="rId342" xr:uid="{DE6E9178-A430-4395-9E7A-540F30BD3DD5}"/>
+    <hyperlink ref="J219" r:id="rId343" xr:uid="{A886421C-9FA0-4D1D-A555-D75C6BBEC56D}"/>
+    <hyperlink ref="K219" r:id="rId344" xr:uid="{03D0F959-65F0-4576-B1C1-EB2A63DAFFFE}"/>
+    <hyperlink ref="L219" r:id="rId345" xr:uid="{83B6EE5F-0FA0-464A-A871-35882B674CD7}"/>
+    <hyperlink ref="M219" r:id="rId346" xr:uid="{20D12798-4F2D-45D8-B3D9-EEDAC8BA81AA}"/>
+    <hyperlink ref="J298" r:id="rId347" xr:uid="{F5527F66-B3DA-41D8-9765-4CA7EEDC97F1}"/>
+    <hyperlink ref="K298" r:id="rId348" xr:uid="{1A2A15F4-5117-42C7-8B70-CA4AB5970A53}"/>
+    <hyperlink ref="L298" r:id="rId349" xr:uid="{9AB03DF6-2293-4BBA-B95F-D4513057928C}"/>
+    <hyperlink ref="M298" r:id="rId350" xr:uid="{A2E339C5-2DF9-4719-964F-F251CB520C94}"/>
+    <hyperlink ref="K61" r:id="rId351" xr:uid="{377B7786-3EAF-416F-99C6-8C77872E4C23}"/>
+    <hyperlink ref="J61" r:id="rId352" xr:uid="{0854386D-6229-4879-9457-DDA376455E76}"/>
+    <hyperlink ref="L61" r:id="rId353" xr:uid="{23628636-C0DC-445A-83E0-3745B69B9189}"/>
+    <hyperlink ref="J200" r:id="rId354" xr:uid="{D0E98960-CCCC-4BE2-BC70-EBA21D7DD8B4}"/>
+    <hyperlink ref="M200" r:id="rId355" xr:uid="{D49963B7-E86C-4490-977A-501B8A78A3DD}"/>
+    <hyperlink ref="J229" r:id="rId356" xr:uid="{87D0FA26-A909-45F1-BD49-F86D89AF1A58}"/>
+    <hyperlink ref="L229" r:id="rId357" xr:uid="{A838D8C4-AC0D-46CD-BEB4-4D5804C43945}"/>
+    <hyperlink ref="K229" r:id="rId358" xr:uid="{D9C5DFF7-9BF6-4BF2-83DC-F549252E49F2}"/>
+    <hyperlink ref="M229" r:id="rId359" xr:uid="{9D3DAEF5-BF30-4D21-916D-450F5C49DEF0}"/>
+    <hyperlink ref="M201" r:id="rId360" xr:uid="{9F7C5EF6-018D-483C-B59B-3DE77ACC60D5}"/>
+    <hyperlink ref="K201" r:id="rId361" xr:uid="{0482AEA3-29E3-4285-BA7C-61171C0896C9}"/>
+    <hyperlink ref="L201" r:id="rId362" xr:uid="{D015EE26-7E89-4DC7-8E92-938B53864255}"/>
+    <hyperlink ref="J201" r:id="rId363" xr:uid="{F3B3A811-947E-4A64-9FD3-9D295407E06F}"/>
+    <hyperlink ref="J141" r:id="rId364" xr:uid="{59736F95-E649-4CFA-8A45-53EF3C5F5FE6}"/>
+    <hyperlink ref="K141" r:id="rId365" xr:uid="{ED28EC78-A0B8-4996-B314-2E390CDDA886}"/>
+    <hyperlink ref="L141" r:id="rId366" xr:uid="{13FC8DC5-72F5-4379-BE4E-9923F5114396}"/>
+    <hyperlink ref="M141" r:id="rId367" xr:uid="{4DB2DF46-3D91-485F-86D1-A018F3AA4C0B}"/>
+    <hyperlink ref="J179" r:id="rId368" xr:uid="{264B41A9-B5FA-48AF-ACB2-AAE3C399AE90}"/>
+    <hyperlink ref="K179" r:id="rId369" xr:uid="{61EE2789-FED2-43B9-A813-328A352754CA}"/>
+    <hyperlink ref="L179" r:id="rId370" xr:uid="{728AEF58-6A7C-4829-A776-9E1F1A2FEC31}"/>
+    <hyperlink ref="M179" r:id="rId371" xr:uid="{1919B1A3-793A-4D63-B5AE-8E4498DDC235}"/>
+    <hyperlink ref="J120" r:id="rId372" xr:uid="{9EED662A-9B0A-42E9-886E-56A9B743EA4A}"/>
+    <hyperlink ref="K120" r:id="rId373" xr:uid="{4EF1B325-BE49-4D6E-9CBD-27713228D023}"/>
+    <hyperlink ref="L120" r:id="rId374" xr:uid="{79D2603C-C10F-4869-8AFD-73E90DC5158A}"/>
+    <hyperlink ref="M120" r:id="rId375" xr:uid="{07C54EF0-2A81-4580-841B-48FE8C5BE427}"/>
+    <hyperlink ref="J202" r:id="rId376" xr:uid="{240A6E84-68A0-4B87-82E1-562572ED7AB7}"/>
+    <hyperlink ref="L202" r:id="rId377" xr:uid="{7BD4B96C-8B86-4D4B-9D11-A81A1AFC1913}"/>
+    <hyperlink ref="M202" r:id="rId378" xr:uid="{69B03112-4BCA-44CA-8AB4-995FF08CC991}"/>
+    <hyperlink ref="J283" r:id="rId379" xr:uid="{3EABF4BD-FDFB-4024-BB99-D5FB80F7420C}"/>
+    <hyperlink ref="M283" r:id="rId380" xr:uid="{8E10395F-6237-4A45-9FAE-9547ED9F3FDB}"/>
+    <hyperlink ref="J203" r:id="rId381" xr:uid="{2FB5AD72-AE18-411D-913F-8A9E4798293B}"/>
+    <hyperlink ref="K203" r:id="rId382" xr:uid="{40BC0523-4BBD-4DC5-8035-5B2FA54C84DD}"/>
+    <hyperlink ref="L203" r:id="rId383" xr:uid="{C103903A-DBC4-4FDD-B63A-AAF14138F219}"/>
+    <hyperlink ref="M203" r:id="rId384" xr:uid="{88D8FF20-9A07-4692-9DA6-7E9441D8853A}"/>
+    <hyperlink ref="J121" r:id="rId385" xr:uid="{CDF21456-7EE7-4FAF-9E29-AC3095E8B710}"/>
+    <hyperlink ref="K121" r:id="rId386" xr:uid="{FB72FBED-F0D8-4EEB-8609-DC41E244C6D5}"/>
+    <hyperlink ref="L121" r:id="rId387" xr:uid="{9FE6BB21-D205-4F42-A4A1-04B7B3B8B867}"/>
+    <hyperlink ref="M121" r:id="rId388" xr:uid="{B259A195-3609-4A06-AC4B-74DA482DE1A8}"/>
+    <hyperlink ref="J180" r:id="rId389" xr:uid="{C432A164-9BBF-401D-A2D8-8A71573C54D8}"/>
+    <hyperlink ref="K180" r:id="rId390" xr:uid="{2D2E3A14-600E-4CFD-8A4E-F0B61820295E}"/>
+    <hyperlink ref="L180" r:id="rId391" xr:uid="{0E159A7A-119E-44FF-A05B-0FFDC2D4E34A}"/>
+    <hyperlink ref="M180" r:id="rId392" xr:uid="{29D68BF5-F2DB-409B-99A9-0CE74D783774}"/>
+    <hyperlink ref="M15" r:id="rId393" xr:uid="{26DC8B78-F5FC-4FFE-9BEB-C68A3D718BF5}"/>
+    <hyperlink ref="J15" r:id="rId394" xr:uid="{36999AC1-13FC-4C81-A5FE-1AE970997895}"/>
+    <hyperlink ref="K15" r:id="rId395" xr:uid="{F1B6CDB3-D7DB-4041-8DA1-36CF172DB220}"/>
+    <hyperlink ref="L15" r:id="rId396" xr:uid="{36074799-65FC-4632-AA92-F02DCCB993A5}"/>
+    <hyperlink ref="J318" r:id="rId397" xr:uid="{7B1640BB-82E7-44A9-BD5B-6FD8C51CC5C4}"/>
+    <hyperlink ref="K318" r:id="rId398" xr:uid="{1BEDE21F-61F4-4AA1-A729-C684C7C4A9A7}"/>
+    <hyperlink ref="L318" r:id="rId399" xr:uid="{626BDFDE-7AC6-43CF-85E2-7D50E0B1B4EC}"/>
+    <hyperlink ref="M318" r:id="rId400" xr:uid="{99EBF6F1-06EB-4315-A3AE-AB9957D3FB2B}"/>
+    <hyperlink ref="M47" r:id="rId401" xr:uid="{7B07B612-3A88-4B60-886F-6FC970BB6B41}"/>
+    <hyperlink ref="J99" r:id="rId402" xr:uid="{0D0C9636-A1BE-4572-9F60-17DA53A1D9B8}"/>
+    <hyperlink ref="K99" r:id="rId403" xr:uid="{73689F04-7E3B-430A-988E-472883578A46}"/>
+    <hyperlink ref="M99" r:id="rId404" xr:uid="{9410E670-EECB-417E-9A31-D3949A0214B2}"/>
+    <hyperlink ref="L99" r:id="rId405" xr:uid="{A215DA8C-109A-4819-9C6D-80C0A1492AC1}"/>
+    <hyperlink ref="J154" r:id="rId406" xr:uid="{8507B41C-7E70-400C-930C-AB114BA6509E}"/>
+    <hyperlink ref="K154" r:id="rId407" xr:uid="{E9FE295A-2D43-420A-8A9E-10F016D11B6C}"/>
+    <hyperlink ref="L154" r:id="rId408" xr:uid="{BE50457E-5FF4-46CE-983A-8A1E71BB846E}"/>
+    <hyperlink ref="M154" r:id="rId409" xr:uid="{5217E048-4675-43D9-9163-562318C43A55}"/>
+    <hyperlink ref="J329" r:id="rId410" xr:uid="{904205CF-7EB6-4895-AFCD-F3B24BB02260}"/>
+    <hyperlink ref="K329" r:id="rId411" xr:uid="{2C2AE4C7-0238-4B56-89D6-B1E30FE2A47E}"/>
+    <hyperlink ref="L329" r:id="rId412" xr:uid="{5F95A1EF-F351-4326-B4B0-0BE11CC3FD81}"/>
+    <hyperlink ref="M329" r:id="rId413" xr:uid="{88820289-C3F9-4DB3-926D-95F74FA46E7F}"/>
+    <hyperlink ref="J181" r:id="rId414" xr:uid="{0DE0D3CC-91C4-48C1-A2B4-EC846B5D1082}"/>
+    <hyperlink ref="K181" r:id="rId415" xr:uid="{B17BCE6D-1CA5-4D3F-9CB9-D26C8358CF7F}"/>
+    <hyperlink ref="L181" r:id="rId416" xr:uid="{ECBAD3DE-BD62-4A89-A694-011DE2D981C1}"/>
+    <hyperlink ref="M181" r:id="rId417" xr:uid="{FDDAB7EC-3DDF-4C42-B006-1E9755E3C809}"/>
+    <hyperlink ref="J68" r:id="rId418" xr:uid="{462837B2-0B52-489B-95BC-8BA6183CC41A}"/>
+    <hyperlink ref="M68" r:id="rId419" xr:uid="{F42FD553-6EB7-4B88-A9FE-261718A340E8}"/>
+    <hyperlink ref="K68" r:id="rId420" xr:uid="{7A183CAD-5D6A-4E1E-A490-A2287DC0528C}"/>
+    <hyperlink ref="L68" r:id="rId421" xr:uid="{B22A6BB4-2BF6-435B-A883-4962FAAAEE8F}"/>
+    <hyperlink ref="J69" r:id="rId422" xr:uid="{F30B54DC-2EEE-4B78-93F0-7E62616FB4DC}"/>
+    <hyperlink ref="M69" r:id="rId423" xr:uid="{B5B739A5-B17C-40F7-8205-0AA4763BC714}"/>
+    <hyperlink ref="I233" r:id="rId424" xr:uid="{C3369525-B7A0-4412-8D59-0C493A78E1DC}"/>
+    <hyperlink ref="J62" r:id="rId425" xr:uid="{E7329603-2EDD-44F0-B789-E1D85A13A5AF}"/>
+    <hyperlink ref="M62" r:id="rId426" xr:uid="{2A04F1A5-411E-4112-96AF-11194F0F7BB9}"/>
+    <hyperlink ref="K62" r:id="rId427" xr:uid="{0386DF53-8D0D-44E0-8911-4355A04799F9}"/>
+    <hyperlink ref="L62" r:id="rId428" xr:uid="{8C766B81-71F9-4A3D-A568-5595B2174541}"/>
+    <hyperlink ref="J98" r:id="rId429" xr:uid="{CF0A4B26-01DE-4363-8D0A-7FDDD09CFCDE}"/>
+    <hyperlink ref="L98" r:id="rId430" xr:uid="{CD04CC97-53AD-43B1-ABAA-2D4FE039CB55}"/>
+    <hyperlink ref="K98" r:id="rId431" xr:uid="{094EBB15-996A-4155-B60F-1048DF22330D}"/>
+    <hyperlink ref="M41" r:id="rId432" xr:uid="{E18AE4E3-ACC6-4772-AF56-2A6606909541}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -27041,16 +27005,16 @@
   <sheetData>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
-        <v>1426</v>
+        <v>1418</v>
       </c>
       <c r="C2" t="s">
-        <v>1427</v>
+        <v>1419</v>
       </c>
       <c r="D2" t="s">
-        <v>1428</v>
+        <v>1420</v>
       </c>
       <c r="E2" t="s">
-        <v>1429</v>
+        <v>1421</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -28710,14 +28674,14 @@
       <c r="F35" s="14"/>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A37" s="33" t="s">
+      <c r="A37" s="34" t="s">
         <v>971</v>
       </c>
-      <c r="B37" s="34"/>
-      <c r="C37" s="34"/>
-      <c r="D37" s="34"/>
-      <c r="E37" s="34"/>
-      <c r="F37" s="34"/>
+      <c r="B37" s="35"/>
+      <c r="C37" s="35"/>
+      <c r="D37" s="35"/>
+      <c r="E37" s="35"/>
+      <c r="F37" s="35"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:F34" xr:uid="{00000000-0009-0000-0000-000003000000}"/>

</xml_diff>